<commit_message>
Fix title typo in index.html and update CT scan and dental templates for improved clarity and consistency
- Corrected the title from "Antesoo Biomedical" to "Anteso Biomedical" in index.html.
- Enhanced the CT scan and dental test data templates by standardizing header formats and improving organization for various tests, including operating potential and radiation output consistency.
- Updated tolerance operators and added new sample rows to enhance clarity in expected results across templates.
</commit_message>
<xml_diff>
--- a/public/templates/CTScan_SingleTube_Sample_updated.xlsx
+++ b/public/templates/CTScan_SingleTube_Sample_updated.xlsx
@@ -397,29 +397,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O77"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:O80"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>TEST: RADIATION PROFILE WIDTH FOR CT SCAN_x000d_</v>
       </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v/>
+      </c>
+      <c r="H1" t="str">
+        <v/>
+      </c>
+      <c r="I1" t="str">
+        <v/>
+      </c>
+      <c r="J1" t="str">
+        <v/>
+      </c>
+      <c r="K1" t="str">
+        <v/>
+      </c>
+      <c r="L1" t="str">
+        <v/>
+      </c>
+      <c r="M1" t="str">
+        <v/>
+      </c>
+      <c r="N1" t="str">
+        <v/>
+      </c>
+      <c r="O1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -434,6 +459,39 @@
       <c r="D2" t="str">
         <v>mA_x000d_</v>
       </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -448,6 +506,39 @@
       <c r="D3" t="str">
         <v>200_x000d_</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -462,6 +553,39 @@
       <c r="D4" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -476,16 +600,133 @@
       <c r="D5" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>TEST: MEASUREMENT OF OPERATING POTENTIAL_x000d_</v>
       </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -515,6 +756,24 @@
       <c r="I8" t="str">
         <v>Tol Sign_x000d_</v>
       </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -544,6 +803,24 @@
       <c r="I9" t="str">
         <v>±_x000d_</v>
       </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -573,6 +850,24 @@
       <c r="I10" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -602,16 +897,118 @@
       <c r="I11" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>TEST: MEASUREMENT OF MA LINEARITY_x000d_</v>
       </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -635,6 +1032,30 @@
       <c r="G14" t="str">
         <v>Meas 3_x000d_</v>
       </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -658,6 +1079,30 @@
       <c r="G15" t="str">
         <v>10.3_x000d_</v>
       </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -681,6 +1126,30 @@
       <c r="G16" t="str">
         <v>20.3_x000d_</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -704,6 +1173,30 @@
       <c r="G17" t="str">
         <v>50.6_x000d_</v>
       </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -727,16 +1220,124 @@
       <c r="G18" t="str">
         <v>101.2_x000d_</v>
       </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
         <v>TEST: TIMER ACCURACY_x000d_</v>
       </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -757,6 +1358,33 @@
       <c r="F21" t="str">
         <v>Tolerance (%)_x000d_</v>
       </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -777,6 +1405,33 @@
       <c r="F22" t="str">
         <v>5_x000d_</v>
       </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -797,16 +1452,127 @@
       <c r="F23" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
         <v>TEST: LINEARITY OF MAS LOADING_x000d_</v>
       </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -824,6 +1590,36 @@
       <c r="E26" t="str">
         <v>Tolerance_x000d_</v>
       </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -841,6 +1637,36 @@
       <c r="E27" t="str">
         <v>0.10_x000d_</v>
       </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -858,16 +1684,130 @@
       <c r="E28" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
         <v>TEST: MEASUREMENT OF CTDI_x000d_</v>
       </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -903,6 +1843,18 @@
       <c r="K31" t="str">
         <v>Body_x000d_</v>
       </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
+      <c r="O31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -938,6 +1890,18 @@
       <c r="K32" t="str">
         <v>13.0_x000d_</v>
       </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+      <c r="O32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -973,6 +1937,18 @@
       <c r="K33" t="str">
         <v>12.5_x000d_</v>
       </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1008,6 +1984,18 @@
       <c r="K34" t="str">
         <v>12.7_x000d_</v>
       </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1042,17 +2030,113 @@
       </c>
       <c r="K35" t="str">
         <v>12.6_x000d_</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
         <v>TEST: TOTAL FILTRATION_x000d_</v>
       </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+      <c r="N37" t="str">
+        <v/>
+      </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1070,6 +2154,36 @@
       <c r="E38" t="str">
         <v>Measured TF_x000d_</v>
       </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1087,206 +2201,293 @@
       <c r="E39" t="str">
         <v>7.5_x000d_</v>
       </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v/>
+      </c>
+      <c r="O39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
         <v>_x000d_</v>
       </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v/>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v/>
+      </c>
+      <c r="O40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
         <v>TEST: Reproducibility of Radiation Output (Consistency Test)_x000d_</v>
       </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v/>
+      </c>
+      <c r="L41" t="str">
+        <v/>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v/>
+      </c>
+      <c r="O41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>mAs</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B42" t="str">
-        <v>Slice Thickness (mm)</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Time (s)</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="E42" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="F42" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="G42" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="H42" t="str">
-        <v>Header 4</v>
-      </c>
-      <c r="I42" t="str">
-        <v>Header 5</v>
-      </c>
-      <c r="J42" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="K42" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="L42" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="M42" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="N42" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="O42" t="str">
-        <v>Meas 5_x000d_</v>
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>100</v>
+        <v>Tolerance Sign</v>
       </c>
       <c r="B43" t="str">
-        <v>5</v>
-      </c>
-      <c r="C43" t="str">
-        <v>1.0</v>
-      </c>
-      <c r="D43" t="str">
-        <v>0.05</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="F43" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="G43" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="I43" t="str">
-        <v>Meas 5</v>
-      </c>
-      <c r="J43" t="str">
-        <v>120</v>
-      </c>
-      <c r="K43" t="str">
-        <v>100.5</v>
-      </c>
-      <c r="L43" t="str">
-        <v>100.3</v>
-      </c>
-      <c r="M43" t="str">
-        <v>100.6</v>
-      </c>
-      <c r="N43" t="str">
-        <v>100.4</v>
-      </c>
-      <c r="O43" t="str">
-        <v>100.5_x000d_</v>
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>_x000d_</v>
+        <v>Tolerance Value (CoV)</v>
+      </c>
+      <c r="B44" t="str">
+        <v>0.05</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>TEST: Radiation Leakage Level from X-Ray Tube House_x000d_</v>
+        <v>mAs</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Slice Thickness (mm)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Time (s)</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Header 4</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Header 5</v>
+      </c>
+      <c r="I45" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="K45" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Meas 4</v>
+      </c>
+      <c r="N45" t="str">
+        <v>Meas 5_x000d_</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>kV</v>
+        <v>100</v>
       </c>
       <c r="B46" t="str">
-        <v>mA</v>
+        <v>5</v>
       </c>
       <c r="C46" t="str">
-        <v>Time (sec)</v>
+        <v>1.0</v>
       </c>
       <c r="D46" t="str">
-        <v>Workload</v>
+        <v>Meas 1</v>
       </c>
       <c r="E46" t="str">
-        <v>Workload Unit</v>
+        <v>Meas 2</v>
       </c>
       <c r="F46" t="str">
-        <v>Tol Value</v>
+        <v>Meas 3</v>
       </c>
       <c r="G46" t="str">
-        <v>Tol Operator</v>
+        <v>Meas 4</v>
       </c>
       <c r="H46" t="str">
-        <v>Tol Time</v>
+        <v>Meas 5</v>
       </c>
       <c r="I46" t="str">
-        <v>Location</v>
+        <v>120</v>
       </c>
       <c r="J46" t="str">
-        <v>Front</v>
+        <v>100.5</v>
       </c>
       <c r="K46" t="str">
-        <v>Back</v>
+        <v>100.3</v>
       </c>
       <c r="L46" t="str">
-        <v>Left</v>
+        <v>100.6</v>
       </c>
       <c r="M46" t="str">
-        <v>Right_x000d_</v>
+        <v>100.4</v>
+      </c>
+      <c r="N46" t="str">
+        <v>100.5_x000d_</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>120</v>
+        <v>_x000d_</v>
       </c>
       <c r="B47" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="C47" t="str">
-        <v>1.0</v>
+        <v/>
       </c>
       <c r="D47" t="str">
-        <v>500</v>
+        <v/>
       </c>
       <c r="E47" t="str">
-        <v>mA·min/week</v>
+        <v/>
       </c>
       <c r="F47" t="str">
-        <v>1.0</v>
+        <v/>
       </c>
       <c r="G47" t="str">
-        <v>less than or equal to</v>
+        <v/>
       </c>
       <c r="H47" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="I47" t="str">
-        <v>Tube</v>
+        <v/>
       </c>
       <c r="J47" t="str">
-        <v>0.05</v>
+        <v/>
       </c>
       <c r="K47" t="str">
-        <v>0.03</v>
+        <v/>
       </c>
       <c r="L47" t="str">
-        <v>0.06</v>
+        <v/>
       </c>
       <c r="M47" t="str">
-        <v>0.04_x000d_</v>
+        <v/>
+      </c>
+      <c r="N47" t="str">
+        <v/>
+      </c>
+      <c r="O47" t="str">
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>TEST: Radiation Leakage Level from X-Ray Tube House_x000d_</v>
       </c>
       <c r="B48" t="str">
         <v/>
@@ -1310,218 +2511,788 @@
         <v/>
       </c>
       <c r="I48" t="str">
-        <v>Collimator</v>
+        <v/>
       </c>
       <c r="J48" t="str">
-        <v>0.02</v>
+        <v/>
       </c>
       <c r="K48" t="str">
-        <v>0.02</v>
+        <v/>
       </c>
       <c r="L48" t="str">
-        <v>0.03</v>
+        <v/>
       </c>
       <c r="M48" t="str">
-        <v>0.01_x000d_</v>
+        <v/>
+      </c>
+      <c r="N48" t="str">
+        <v/>
+      </c>
+      <c r="O48" t="str">
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>_x000d_</v>
+        <v>kV</v>
+      </c>
+      <c r="B49" t="str">
+        <v>mA</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Time (sec)</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Workload</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Workload Unit</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Tol Value</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Tol Operator</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Tol Time</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Location</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Front</v>
+      </c>
+      <c r="K49" t="str">
+        <v>Back</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M49" t="str">
+        <v>Right_x000d_</v>
+      </c>
+      <c r="N49" t="str">
+        <v/>
+      </c>
+      <c r="O49" t="str">
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION_x000d_</v>
+        <v>120</v>
+      </c>
+      <c r="B50" t="str">
+        <v>100</v>
+      </c>
+      <c r="C50" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="D50" t="str">
+        <v>500</v>
+      </c>
+      <c r="E50" t="str">
+        <v>mA·min/week</v>
+      </c>
+      <c r="F50" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="G50" t="str">
+        <v>less than or equal to</v>
+      </c>
+      <c r="H50" t="str">
+        <v>1</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="J50" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="K50" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="L50" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="M50" t="str">
+        <v>0.04_x000d_</v>
+      </c>
+      <c r="N50" t="str">
+        <v/>
+      </c>
+      <c r="O50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Observed Size</v>
+        <v/>
       </c>
       <c r="B51" t="str">
-        <v>Contrast Level</v>
+        <v/>
       </c>
       <c r="C51" t="str">
-        <v>kVp</v>
+        <v/>
       </c>
       <c r="D51" t="str">
-        <v>mA</v>
+        <v/>
       </c>
       <c r="E51" t="str">
-        <v>Slice Thickness</v>
+        <v/>
       </c>
       <c r="F51" t="str">
-        <v>WW_x000d_</v>
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v>Collimator</v>
+      </c>
+      <c r="J51" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="K51" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="L51" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="M51" t="str">
+        <v>0.01_x000d_</v>
+      </c>
+      <c r="N51" t="str">
+        <v/>
+      </c>
+      <c r="O51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>3.0</v>
+        <v>_x000d_</v>
       </c>
       <c r="B52" t="str">
-        <v>1.0</v>
+        <v/>
       </c>
       <c r="C52" t="str">
-        <v>120</v>
+        <v/>
       </c>
       <c r="D52" t="str">
-        <v>200</v>
+        <v/>
       </c>
       <c r="E52" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="F52" t="str">
-        <v>400_x000d_</v>
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v/>
+      </c>
+      <c r="L52" t="str">
+        <v/>
+      </c>
+      <c r="M52" t="str">
+        <v/>
+      </c>
+      <c r="N52" t="str">
+        <v/>
+      </c>
+      <c r="O52" t="str">
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>_x000d_</v>
+        <v>TEST: LOW CONTRAST RESOLUTION_x000d_</v>
+      </c>
+      <c r="B53" t="str">
+        <v/>
+      </c>
+      <c r="C53" t="str">
+        <v/>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v/>
+      </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
+        <v/>
+      </c>
+      <c r="N53" t="str">
+        <v/>
+      </c>
+      <c r="O53" t="str">
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION_x000d_</v>
+        <v>Observed Size</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Contrast Level</v>
+      </c>
+      <c r="C54" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="D54" t="str">
+        <v>mA</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Slice Thickness</v>
+      </c>
+      <c r="F54" t="str">
+        <v>WW_x000d_</v>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
+        <v/>
+      </c>
+      <c r="L54" t="str">
+        <v/>
+      </c>
+      <c r="M54" t="str">
+        <v/>
+      </c>
+      <c r="N54" t="str">
+        <v/>
+      </c>
+      <c r="O54" t="str">
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Observed Size</v>
+        <v>3.0</v>
       </c>
       <c r="B55" t="str">
-        <v>Contrast Difference</v>
+        <v>1.0</v>
       </c>
       <c r="C55" t="str">
-        <v>kVp</v>
+        <v>120</v>
       </c>
       <c r="D55" t="str">
-        <v>mAs</v>
+        <v>200</v>
       </c>
       <c r="E55" t="str">
-        <v>Slice Thickness</v>
+        <v>5</v>
       </c>
       <c r="F55" t="str">
-        <v>WW_x000d_</v>
+        <v>400_x000d_</v>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v/>
+      </c>
+      <c r="L55" t="str">
+        <v/>
+      </c>
+      <c r="M55" t="str">
+        <v/>
+      </c>
+      <c r="N55" t="str">
+        <v/>
+      </c>
+      <c r="O55" t="str">
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>0.5</v>
+        <v>_x000d_</v>
       </c>
       <c r="B56" t="str">
-        <v>5.0</v>
+        <v/>
       </c>
       <c r="C56" t="str">
-        <v>120</v>
+        <v/>
       </c>
       <c r="D56" t="str">
-        <v>200</v>
+        <v/>
       </c>
       <c r="E56" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="F56" t="str">
-        <v>400_x000d_</v>
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v/>
+      </c>
+      <c r="L56" t="str">
+        <v/>
+      </c>
+      <c r="M56" t="str">
+        <v/>
+      </c>
+      <c r="N56" t="str">
+        <v/>
+      </c>
+      <c r="O56" t="str">
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>_x000d_</v>
+        <v>TEST: HIGH CONTRAST RESOLUTION_x000d_</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v/>
+      </c>
+      <c r="L57" t="str">
+        <v/>
+      </c>
+      <c r="M57" t="str">
+        <v/>
+      </c>
+      <c r="N57" t="str">
+        <v/>
+      </c>
+      <c r="O57" t="str">
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>TEST: ALIGNMENT OF TABLE/GANTRY_x000d_</v>
+        <v>Observed Size</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Contrast Difference</v>
+      </c>
+      <c r="C58" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="D58" t="str">
+        <v>mAs</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Slice Thickness</v>
+      </c>
+      <c r="F58" t="str">
+        <v>WW_x000d_</v>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
+        <v/>
+      </c>
+      <c r="L58" t="str">
+        <v/>
+      </c>
+      <c r="M58" t="str">
+        <v/>
+      </c>
+      <c r="N58" t="str">
+        <v/>
+      </c>
+      <c r="O58" t="str">
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Result</v>
+        <v>0.5</v>
       </c>
       <c r="B59" t="str">
-        <v>Tolerance_x000d_</v>
+        <v>5.0</v>
+      </c>
+      <c r="C59" t="str">
+        <v>120</v>
+      </c>
+      <c r="D59" t="str">
+        <v>200</v>
+      </c>
+      <c r="E59" t="str">
+        <v>5</v>
+      </c>
+      <c r="F59" t="str">
+        <v>400_x000d_</v>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
+        <v/>
+      </c>
+      <c r="L59" t="str">
+        <v/>
+      </c>
+      <c r="M59" t="str">
+        <v/>
+      </c>
+      <c r="N59" t="str">
+        <v/>
+      </c>
+      <c r="O59" t="str">
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2.0</v>
+        <v>_x000d_</v>
       </c>
       <c r="B60" t="str">
-        <v>±2.0_x000d_</v>
+        <v/>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+      <c r="K60" t="str">
+        <v/>
+      </c>
+      <c r="L60" t="str">
+        <v/>
+      </c>
+      <c r="M60" t="str">
+        <v/>
+      </c>
+      <c r="N60" t="str">
+        <v/>
+      </c>
+      <c r="O60" t="str">
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>_x000d_</v>
+        <v>TEST: ALIGNMENT OF TABLE/GANTRY_x000d_</v>
+      </c>
+      <c r="B61" t="str">
+        <v/>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
+        <v/>
+      </c>
+      <c r="L61" t="str">
+        <v/>
+      </c>
+      <c r="M61" t="str">
+        <v/>
+      </c>
+      <c r="N61" t="str">
+        <v/>
+      </c>
+      <c r="O61" t="str">
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>TEST: TABLE POSITION_x000d_</v>
+        <v>Result</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Tolerance_x000d_</v>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
+        <v/>
+      </c>
+      <c r="L62" t="str">
+        <v/>
+      </c>
+      <c r="M62" t="str">
+        <v/>
+      </c>
+      <c r="N62" t="str">
+        <v/>
+      </c>
+      <c r="O62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Table Position</v>
+        <v>2.0</v>
       </c>
       <c r="B63" t="str">
-        <v>Expected</v>
+        <v>±2.0_x000d_</v>
       </c>
       <c r="C63" t="str">
-        <v>Measured</v>
+        <v/>
       </c>
       <c r="D63" t="str">
-        <v>Initial Pos</v>
+        <v/>
       </c>
       <c r="E63" t="str">
-        <v>Load</v>
+        <v/>
       </c>
       <c r="F63" t="str">
-        <v>kVp</v>
+        <v/>
       </c>
       <c r="G63" t="str">
-        <v>mA</v>
+        <v/>
       </c>
       <c r="H63" t="str">
-        <v>Slice Thickness_x000d_</v>
+        <v/>
+      </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
+        <v/>
+      </c>
+      <c r="L63" t="str">
+        <v/>
+      </c>
+      <c r="M63" t="str">
+        <v/>
+      </c>
+      <c r="N63" t="str">
+        <v/>
+      </c>
+      <c r="O63" t="str">
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>10</v>
+        <v>_x000d_</v>
       </c>
       <c r="B64" t="str">
-        <v>10</v>
+        <v/>
       </c>
       <c r="C64" t="str">
-        <v>10.1</v>
+        <v/>
       </c>
       <c r="D64" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="E64" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="F64" t="str">
-        <v>120</v>
+        <v/>
       </c>
       <c r="G64" t="str">
-        <v>200</v>
+        <v/>
       </c>
       <c r="H64" t="str">
-        <v>5.0_x000d_</v>
+        <v/>
+      </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
+        <v/>
+      </c>
+      <c r="L64" t="str">
+        <v/>
+      </c>
+      <c r="M64" t="str">
+        <v/>
+      </c>
+      <c r="N64" t="str">
+        <v/>
+      </c>
+      <c r="O64" t="str">
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>20</v>
+        <v>TEST: TABLE POSITION_x000d_</v>
       </c>
       <c r="B65" t="str">
-        <v>20</v>
+        <v/>
       </c>
       <c r="C65" t="str">
-        <v>19.9</v>
+        <v/>
       </c>
       <c r="D65" t="str">
         <v/>
@@ -1536,140 +3307,509 @@
         <v/>
       </c>
       <c r="H65" t="str">
-        <v>_x000d_</v>
+        <v/>
+      </c>
+      <c r="I65" t="str">
+        <v/>
+      </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
+      <c r="K65" t="str">
+        <v/>
+      </c>
+      <c r="L65" t="str">
+        <v/>
+      </c>
+      <c r="M65" t="str">
+        <v/>
+      </c>
+      <c r="N65" t="str">
+        <v/>
+      </c>
+      <c r="O65" t="str">
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>_x000d_</v>
+        <v>Table Position</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Expected</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Measured</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Initial Pos</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Load</v>
+      </c>
+      <c r="F66" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="G66" t="str">
+        <v>mA</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Slice Thickness_x000d_</v>
+      </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
+      <c r="K66" t="str">
+        <v/>
+      </c>
+      <c r="L66" t="str">
+        <v/>
+      </c>
+      <c r="M66" t="str">
+        <v/>
+      </c>
+      <c r="N66" t="str">
+        <v/>
+      </c>
+      <c r="O66" t="str">
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>TEST: GANTRY TILT_x000d_</v>
+        <v>10</v>
+      </c>
+      <c r="B67" t="str">
+        <v>10</v>
+      </c>
+      <c r="C67" t="str">
+        <v>10.1</v>
+      </c>
+      <c r="D67" t="str">
+        <v>0</v>
+      </c>
+      <c r="E67" t="str">
+        <v>100</v>
+      </c>
+      <c r="F67" t="str">
+        <v>120</v>
+      </c>
+      <c r="G67" t="str">
+        <v>200</v>
+      </c>
+      <c r="H67" t="str">
+        <v>5.0_x000d_</v>
+      </c>
+      <c r="I67" t="str">
+        <v/>
+      </c>
+      <c r="J67" t="str">
+        <v/>
+      </c>
+      <c r="K67" t="str">
+        <v/>
+      </c>
+      <c r="L67" t="str">
+        <v/>
+      </c>
+      <c r="M67" t="str">
+        <v/>
+      </c>
+      <c r="N67" t="str">
+        <v/>
+      </c>
+      <c r="O67" t="str">
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Type</v>
+        <v>20</v>
       </c>
       <c r="B68" t="str">
-        <v>Name/Actual</v>
+        <v>20</v>
       </c>
       <c r="C68" t="str">
-        <v>Value/Measured_x000d_</v>
+        <v>19.9</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
+      <c r="H68" t="str">
+        <v>_x000d_</v>
+      </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
+      <c r="J68" t="str">
+        <v/>
+      </c>
+      <c r="K68" t="str">
+        <v/>
+      </c>
+      <c r="L68" t="str">
+        <v/>
+      </c>
+      <c r="M68" t="str">
+        <v/>
+      </c>
+      <c r="N68" t="str">
+        <v/>
+      </c>
+      <c r="O68" t="str">
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Parameter</v>
+        <v>_x000d_</v>
       </c>
       <c r="B69" t="str">
-        <v>Tilt Param</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>45_x000d_</v>
+        <v/>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
+      <c r="I69" t="str">
+        <v/>
+      </c>
+      <c r="J69" t="str">
+        <v/>
+      </c>
+      <c r="K69" t="str">
+        <v/>
+      </c>
+      <c r="L69" t="str">
+        <v/>
+      </c>
+      <c r="M69" t="str">
+        <v/>
+      </c>
+      <c r="N69" t="str">
+        <v/>
+      </c>
+      <c r="O69" t="str">
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Measurement</v>
+        <v>TEST: GANTRY TILT_x000d_</v>
       </c>
       <c r="B70" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="C70" t="str">
-        <v>0.5_x000d_</v>
+        <v/>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
+      <c r="J70" t="str">
+        <v/>
+      </c>
+      <c r="K70" t="str">
+        <v/>
+      </c>
+      <c r="L70" t="str">
+        <v/>
+      </c>
+      <c r="M70" t="str">
+        <v/>
+      </c>
+      <c r="N70" t="str">
+        <v/>
+      </c>
+      <c r="O70" t="str">
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Measurement</v>
+        <v>Type</v>
       </c>
       <c r="B71" t="str">
-        <v>30</v>
+        <v>Name/Actual</v>
       </c>
       <c r="C71" t="str">
-        <v>30.2_x000d_</v>
+        <v>Value/Measured_x000d_</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
+      <c r="J71" t="str">
+        <v/>
+      </c>
+      <c r="K71" t="str">
+        <v/>
+      </c>
+      <c r="L71" t="str">
+        <v/>
+      </c>
+      <c r="M71" t="str">
+        <v/>
+      </c>
+      <c r="N71" t="str">
+        <v/>
+      </c>
+      <c r="O71" t="str">
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>_x000d_</v>
+        <v>Parameter</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Tilt Param</v>
+      </c>
+      <c r="C72" t="str">
+        <v>45_x000d_</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
+      <c r="H72" t="str">
+        <v/>
+      </c>
+      <c r="I72" t="str">
+        <v/>
+      </c>
+      <c r="J72" t="str">
+        <v/>
+      </c>
+      <c r="K72" t="str">
+        <v/>
+      </c>
+      <c r="L72" t="str">
+        <v/>
+      </c>
+      <c r="M72" t="str">
+        <v/>
+      </c>
+      <c r="N72" t="str">
+        <v/>
+      </c>
+      <c r="O72" t="str">
+        <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>TEST: MAXIMUM RADIATION LEVEL_x000d_</v>
+        <v>Measurement</v>
+      </c>
+      <c r="B73" t="str">
+        <v>0</v>
+      </c>
+      <c r="C73" t="str">
+        <v>0.5_x000d_</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
+      <c r="J73" t="str">
+        <v/>
+      </c>
+      <c r="K73" t="str">
+        <v/>
+      </c>
+      <c r="L73" t="str">
+        <v/>
+      </c>
+      <c r="M73" t="str">
+        <v/>
+      </c>
+      <c r="N73" t="str">
+        <v/>
+      </c>
+      <c r="O73" t="str">
+        <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Location</v>
+        <v>Measurement</v>
       </c>
       <c r="B74" t="str">
-        <v>mR/hr</v>
+        <v>30</v>
       </c>
       <c r="C74" t="str">
-        <v>Category</v>
+        <v>30.2_x000d_</v>
       </c>
       <c r="D74" t="str">
-        <v>Date</v>
+        <v/>
       </c>
       <c r="E74" t="str">
-        <v>Calibrated</v>
+        <v/>
       </c>
       <c r="F74" t="str">
-        <v>mA</v>
+        <v/>
       </c>
       <c r="G74" t="str">
-        <v>kV</v>
+        <v/>
       </c>
       <c r="H74" t="str">
-        <v>Time</v>
+        <v/>
       </c>
       <c r="I74" t="str">
-        <v>Workload_x000d_</v>
+        <v/>
+      </c>
+      <c r="J74" t="str">
+        <v/>
+      </c>
+      <c r="K74" t="str">
+        <v/>
+      </c>
+      <c r="L74" t="str">
+        <v/>
+      </c>
+      <c r="M74" t="str">
+        <v/>
+      </c>
+      <c r="N74" t="str">
+        <v/>
+      </c>
+      <c r="O74" t="str">
+        <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Control Console</v>
+        <v>_x000d_</v>
       </c>
       <c r="B75" t="str">
-        <v>0.02</v>
+        <v/>
       </c>
       <c r="C75" t="str">
-        <v>worker</v>
+        <v/>
       </c>
       <c r="D75" t="str">
-        <v>2024-01-01</v>
+        <v/>
       </c>
       <c r="E75" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="F75" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="G75" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="H75" t="str">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="I75" t="str">
-        <v>5000_x000d_</v>
+        <v/>
+      </c>
+      <c r="J75" t="str">
+        <v/>
+      </c>
+      <c r="K75" t="str">
+        <v/>
+      </c>
+      <c r="L75" t="str">
+        <v/>
+      </c>
+      <c r="M75" t="str">
+        <v/>
+      </c>
+      <c r="N75" t="str">
+        <v/>
+      </c>
+      <c r="O75" t="str">
+        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Patient Entrance Door</v>
+        <v>TEST: MAXIMUM RADIATION LEVEL_x000d_</v>
       </c>
       <c r="B76" t="str">
-        <v>0.05</v>
+        <v/>
       </c>
       <c r="C76" t="str">
-        <v>worker</v>
+        <v/>
       </c>
       <c r="D76" t="str">
         <v/>
@@ -1687,17 +3827,218 @@
         <v/>
       </c>
       <c r="I76" t="str">
-        <v>_x000d_</v>
+        <v/>
+      </c>
+      <c r="J76" t="str">
+        <v/>
+      </c>
+      <c r="K76" t="str">
+        <v/>
+      </c>
+      <c r="L76" t="str">
+        <v/>
+      </c>
+      <c r="M76" t="str">
+        <v/>
+      </c>
+      <c r="N76" t="str">
+        <v/>
+      </c>
+      <c r="O76" t="str">
+        <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
+        <v>Location</v>
+      </c>
+      <c r="B77" t="str">
+        <v>mR/hr</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Date</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Calibrated</v>
+      </c>
+      <c r="F77" t="str">
+        <v>mA</v>
+      </c>
+      <c r="G77" t="str">
+        <v>kV</v>
+      </c>
+      <c r="H77" t="str">
+        <v>Time</v>
+      </c>
+      <c r="I77" t="str">
+        <v>Workload_x000d_</v>
+      </c>
+      <c r="J77" t="str">
+        <v/>
+      </c>
+      <c r="K77" t="str">
+        <v/>
+      </c>
+      <c r="L77" t="str">
+        <v/>
+      </c>
+      <c r="M77" t="str">
+        <v/>
+      </c>
+      <c r="N77" t="str">
+        <v/>
+      </c>
+      <c r="O77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Control Console</v>
+      </c>
+      <c r="B78" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="C78" t="str">
+        <v>worker</v>
+      </c>
+      <c r="D78" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F78" t="str">
+        <v>100</v>
+      </c>
+      <c r="G78" t="str">
+        <v>80</v>
+      </c>
+      <c r="H78" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="I78" t="str">
+        <v>5000_x000d_</v>
+      </c>
+      <c r="J78" t="str">
+        <v/>
+      </c>
+      <c r="K78" t="str">
+        <v/>
+      </c>
+      <c r="L78" t="str">
+        <v/>
+      </c>
+      <c r="M78" t="str">
+        <v/>
+      </c>
+      <c r="N78" t="str">
+        <v/>
+      </c>
+      <c r="O78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Patient Entrance Door</v>
+      </c>
+      <c r="B79" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="C79" t="str">
+        <v>worker</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v>_x000d_</v>
+      </c>
+      <c r="J79" t="str">
+        <v/>
+      </c>
+      <c r="K79" t="str">
+        <v/>
+      </c>
+      <c r="L79" t="str">
+        <v/>
+      </c>
+      <c r="M79" t="str">
+        <v/>
+      </c>
+      <c r="N79" t="str">
+        <v/>
+      </c>
+      <c r="O79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v/>
+      </c>
+      <c r="B80" t="str">
+        <v/>
+      </c>
+      <c r="C80" t="str">
+        <v/>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+      <c r="I80" t="str">
+        <v/>
+      </c>
+      <c r="J80" t="str">
+        <v/>
+      </c>
+      <c r="K80" t="str">
+        <v/>
+      </c>
+      <c r="L80" t="str">
+        <v/>
+      </c>
+      <c r="M80" t="str">
+        <v/>
+      </c>
+      <c r="N80" t="str">
+        <v/>
+      </c>
+      <c r="O80" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O80"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>